<commit_message>
[20260310_115400_vd_ingame_masterdata_generation] ブロック基礎設計xlsx再生成 vd_aya_normal_00001 / vd_aya_boss_00001 / vd_chi_normal_00001 / vd_chi_boss_00001 / vd_gom_normal_00001
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/domain/tasks/20260310_115400_vd_ingame_masterdata_generation/vd-ingame-creator/vd_aya_boss_00001/vd_aya_boss_00001.xlsx
+++ b/domain/tasks/20260310_115400_vd_ingame_masterdata_generation/vd-ingame-creator/vd_aya_boss_00001/vd_aya_boss_00001.xlsx
@@ -980,7 +980,11 @@
           <t>1コマ</t>
         </is>
       </c>
-      <c r="D14" s="26" t="inlineStr"/>
+      <c r="D14" s="26" t="inlineStr">
+        <is>
+          <t>aya_00002</t>
+        </is>
+      </c>
       <c r="E14" s="26" t="inlineStr">
         <is>
           <t>None</t>
@@ -988,7 +992,7 @@
       </c>
       <c r="F14" s="26" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1.00</t>
         </is>
       </c>
       <c r="G14" s="2" t="n"/>
@@ -1245,7 +1249,7 @@
       </c>
       <c r="I26" s="26" t="inlineStr">
         <is>
-          <t>ボス</t>
+          <t>ボス（c_キャラ）</t>
         </is>
       </c>
       <c r="J26" s="2" t="n"/>
@@ -1286,7 +1290,7 @@
       </c>
       <c r="I27" s="26" t="inlineStr">
         <is>
-          <t>雑魚</t>
+          <t>雑魚（e_キャラ）</t>
         </is>
       </c>
       <c r="J27" s="2" t="n"/>
@@ -1560,7 +1564,7 @@
       </c>
       <c r="H40" s="26" t="inlineStr">
         <is>
-          <t>ボス・summon_position=1.7・Boss オーラ</t>
+          <t>開幕ボス・summon_position=1.7・Bossオーラ・Damage 1で進軍</t>
         </is>
       </c>
       <c r="I40" s="2" t="n"/>
@@ -1597,7 +1601,7 @@
       </c>
       <c r="H41" s="26" t="inlineStr">
         <is>
-          <t>summon_interval=1500ms</t>
+          <t>3体・summon_interval=1500ms・時間差出現</t>
         </is>
       </c>
       <c r="I41" s="2" t="n"/>
@@ -1632,7 +1636,11 @@
       <c r="G42" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="H42" s="26" t="inlineStr"/>
+      <c r="H42" s="26" t="inlineStr">
+        <is>
+          <t>3体追加・合計7体</t>
+        </is>
+      </c>
       <c r="I42" s="2" t="n"/>
       <c r="J42" s="2" t="n"/>
       <c r="K42" s="2" t="n"/>
@@ -1883,7 +1891,7 @@
           <t>バトルヒント</t>
         </is>
       </c>
-      <c r="C58" s="26" t="inlineStr"/>
+      <c r="C58" s="18" t="inlineStr"/>
       <c r="D58" s="27" t="n"/>
       <c r="E58" s="27" t="n"/>
       <c r="F58" s="27" t="n"/>
@@ -1902,7 +1910,7 @@
           <t>ステージ説明文</t>
         </is>
       </c>
-      <c r="C59" s="26" t="inlineStr"/>
+      <c r="C59" s="18" t="inlineStr"/>
       <c r="D59" s="27" t="n"/>
       <c r="E59" s="27" t="n"/>
       <c r="F59" s="27" t="n"/>
@@ -2242,7 +2250,11 @@
         </is>
       </c>
       <c r="M2" s="31" t="inlineStr"/>
-      <c r="N2" s="31" t="inlineStr"/>
+      <c r="N2" s="31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="O2" s="31" t="inlineStr">
         <is>
           <t>1.7</t>
@@ -2258,9 +2270,17 @@
           <t>1</t>
         </is>
       </c>
-      <c r="R2" s="31" t="inlineStr"/>
+      <c r="R2" s="31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="S2" s="31" t="inlineStr"/>
-      <c r="T2" s="31" t="inlineStr"/>
+      <c r="T2" s="31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="U2" s="31" t="inlineStr"/>
       <c r="V2" s="31" t="inlineStr"/>
       <c r="W2" s="31" t="inlineStr"/>
@@ -2270,7 +2290,11 @@
           <t>Boss</t>
         </is>
       </c>
-      <c r="Z2" s="31" t="inlineStr"/>
+      <c r="Z2" s="31" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
       <c r="AA2" s="31" t="inlineStr">
         <is>
           <t>1</t>
@@ -2287,9 +2311,17 @@
         </is>
       </c>
       <c r="AD2" s="31" t="inlineStr"/>
-      <c r="AE2" s="31" t="inlineStr"/>
+      <c r="AE2" s="31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="AF2" s="31" t="inlineStr"/>
-      <c r="AG2" s="31" t="inlineStr"/>
+      <c r="AG2" s="31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="AH2" s="31" t="inlineStr"/>
       <c r="AI2" s="31" t="inlineStr">
         <is>
@@ -2351,13 +2383,29 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="N3" s="31" t="inlineStr"/>
+      <c r="N3" s="31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="O3" s="31" t="inlineStr"/>
-      <c r="P3" s="31" t="inlineStr"/>
+      <c r="P3" s="31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="Q3" s="31" t="inlineStr"/>
-      <c r="R3" s="31" t="inlineStr"/>
+      <c r="R3" s="31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="S3" s="31" t="inlineStr"/>
-      <c r="T3" s="31" t="inlineStr"/>
+      <c r="T3" s="31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="U3" s="31" t="inlineStr"/>
       <c r="V3" s="31" t="inlineStr"/>
       <c r="W3" s="31" t="inlineStr"/>
@@ -2384,9 +2432,17 @@
           <t>1</t>
         </is>
       </c>
-      <c r="AE3" s="31" t="inlineStr"/>
+      <c r="AE3" s="31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="AF3" s="31" t="inlineStr"/>
-      <c r="AG3" s="31" t="inlineStr"/>
+      <c r="AG3" s="31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="AH3" s="31" t="inlineStr"/>
       <c r="AI3" s="31" t="inlineStr"/>
       <c r="AJ3" s="31" t="inlineStr">
@@ -2445,13 +2501,29 @@
         </is>
       </c>
       <c r="M4" s="31" t="inlineStr"/>
-      <c r="N4" s="31" t="inlineStr"/>
+      <c r="N4" s="31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="O4" s="31" t="inlineStr"/>
-      <c r="P4" s="31" t="inlineStr"/>
+      <c r="P4" s="31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="Q4" s="31" t="inlineStr"/>
-      <c r="R4" s="31" t="inlineStr"/>
+      <c r="R4" s="31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="S4" s="31" t="inlineStr"/>
-      <c r="T4" s="31" t="inlineStr"/>
+      <c r="T4" s="31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="U4" s="31" t="inlineStr"/>
       <c r="V4" s="31" t="inlineStr"/>
       <c r="W4" s="31" t="inlineStr"/>
@@ -2461,7 +2533,11 @@
           <t>Default</t>
         </is>
       </c>
-      <c r="Z4" s="31" t="inlineStr"/>
+      <c r="Z4" s="31" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
       <c r="AA4" s="31" t="inlineStr">
         <is>
           <t>1</t>
@@ -2478,9 +2554,17 @@
         </is>
       </c>
       <c r="AD4" s="31" t="inlineStr"/>
-      <c r="AE4" s="31" t="inlineStr"/>
+      <c r="AE4" s="31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="AF4" s="31" t="inlineStr"/>
-      <c r="AG4" s="31" t="inlineStr"/>
+      <c r="AG4" s="31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="AH4" s="31" t="inlineStr"/>
       <c r="AI4" s="31" t="inlineStr">
         <is>
@@ -3402,13 +3486,21 @@
         </is>
       </c>
       <c r="F2" s="31" t="inlineStr"/>
-      <c r="G2" s="31" t="inlineStr"/>
+      <c r="G2" s="31" t="inlineStr">
+        <is>
+          <t>aya_00002</t>
+        </is>
+      </c>
       <c r="H2" s="31" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="I2" s="31" t="inlineStr"/>
+      <c r="I2" s="31" t="inlineStr">
+        <is>
+          <t>-1.0</t>
+        </is>
+      </c>
       <c r="J2" s="31" t="inlineStr">
         <is>
           <t>None</t>

</xml_diff>